<commit_message>
Add 21 new golf, F&B, leisure and geographic-diversity programmes
Closes the "no private/reciprocal clubs" gap in Golf (9 clubs including
Eligo, Troon Privé, PlatinumClubNet), the 0%-Premium/Luxury gap in Food &
Beverage (7 private members' clubs and curated subscriptions) and in
Leisure & Entertainment (Yellowstone Club), plus 4 programmes headquartered
outside the US/UK/Portugal/Western-Europe cluster that dominates the
existing sample (Neera, Capital Club Dubai, Rotana DISCOVERY, Zomato Gold).

Appends the 21 rows to the staging workbook and adds the Supabase insert
script (migration/add_new_programmes_2026_batch2.py) — not yet run against
the live database, since this environment's network policy blocks
dyuflyhkanmczwshmbyh.supabase.co.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013D2DpzkAdSZ9P2CkDZucfZ
</commit_message>
<xml_diff>
--- a/migration/Details_Loyalty_Staging_Workbook.xlsx
+++ b/migration/Details_Loyalty_Staging_Workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28160" windowHeight="17620" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROGRAMMES" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIERS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FEATURES" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PICK LISTS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PROGRAMMES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TIERS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FEATURES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PICK LISTS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dictionary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="AccessReg_List">'PICK LISTS'!$H$4:$H$8</definedName>
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U207"/>
+  <dimension ref="A1:U228"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="14" min="1" max="1"/>
@@ -18232,6 +18232,1348 @@
       <c r="U207" t="inlineStr">
         <is>
           <t>https://tiff.net/membership</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Vilamoura Golf Membership</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Vilamoura Golf</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>https://www.vilamouragolf.com/wp-content/uploads/2025/02/VM-Golf-Logo-Slate-Green-RGB.png</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Enthusiasts / Hobbyists; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>Member pricing; Privileged access; Included member benefits</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>https://www.vilamouragolf.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Golf Club Membership</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Golf Club</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Resort</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcScsGWEwTQ0yq4jNdzWjJ3NTOHbAygD1i-Aeoe3MIPiRKmfqTULFowr-fsI&amp;s=10</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; Enthusiasts / Hobbyists</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>Member pricing; Privileged access; Included member benefits</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>https://www.valedolobo.com/wp-content/uploads/2025/01/2025_Golf_Club_Membership.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Amendoeira Golf Resort Membership</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Amendoeira Golf Resort</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcT4sVOPTInd3Y_LcwZgd0TAZl-NQt6wnPONehLhgbBicyYowKJW9kgBRmY&amp;s=10</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Enthusiasts / Hobbyists</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>Open registration</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>Member pricing; Privileged access</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>https://www.amendoeiraresort.com/en/golf/</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Monte Rei Golf &amp; Country Club</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Monte Rei Golf &amp; Country Club</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQIx2SWFzivpIg-WNpI4Ptfpj0mXl2cn4IwyAtv778VwvRzmA51SmdFsxug&amp;s=10</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; Enthusiasts / Hobbyists</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>Privileged access; Member experiences &amp; events; Community; Included member benefits</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>https://www.monte-rei.com/en/golf/</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Eligo Club</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Eligo Club</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>https://p-gpb8fhd4b9fbh6fy.z01.azurefd.net/logos/209086c0-e6fe-4498-877b-964cac90e4ab/medium.png</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Enthusiasts / Hobbyists; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Europe; North America</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>External partner network; Privileged access; Member experiences &amp; events; Community</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>https://www.eligoclub.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Troon Privé (Private Club Golf)</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Troon</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>https://www.oakspga.cz/wp-content/uploads/sites/9225/2023/08/TroonPrivilegesLogo-1.png?w=1024</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Enthusiasts / Hobbyists; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>External partner network; Privileged access; Member pricing</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>https://troon.com/member-programs/private-club-golf</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>PlatinumClubNet</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>PlatinumClubNet</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>MobiCom America Inc.</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>https://www.platinumclubnet.com/_next/image?url=%2F_next%2Fstatic%2Fmedia%2Flog1.73b78c22.png&amp;w=256&amp;q=75</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>High-Value Customers; Premium / Luxury Customers</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>Invitation only</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>External partner network; Privileged access; Community</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>https://www.platinumclubnet.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Les Bordes Golf Club</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Les Bordes Golf Club</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>https://golfcoursegurus.com/reviews/images/logos/Les-Bordes-Golf-Club-New.png</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; Enthusiasts / Hobbyists</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>Privileged access; Community; Member experiences &amp; events; Included member benefits</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>https://www.lesbordesgolfclub.com/club/membership/</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Queenwood Golf Club</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Queenwood Golf Club</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/C560BAQH6rhMQDhVYgw/company-logo_200_200/company-logo_200_200/0/1630610259895/queenwood_golf_club_limited_logo?e=2147483647&amp;v=beta&amp;t=5UeZPLDRJIY2irAJfir_jEahHJvCVRwAHD_n3hifeSk</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Golf</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Invitation only</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>Privileged access; Community; Member experiences &amp; events</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Queenwood_Golf_Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>JNcQUOI Club</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>JNcQUOI</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Amorim Luxury</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>https://www.visitgrandola.com/cmgrandola/uploads/poi/image/995/jncquoi.JPG</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; International Customers</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>Member pricing; Privileged access; Included member benefits; Member experiences &amp; events</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>https://www.jncquoi.com/en/membership/</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Soho House</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Soho House &amp; Co</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/d3/94/ca/d394ca792d0594d99eb16795dfa0c73a.jpg</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; International Customers</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Subscription</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>Community; Privileged access; Member experiences &amp; events; Included member benefits; Ecosystem cross-use</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>https://www.sohohouse.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Annabel's (Birley Clubs)</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Annabel's</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Birley Clubs</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>https://storage.googleapis.com/talentfunnel-cms-career-site-storage/birley-clubs/Annabels_2_842f94c806_bfb48f2e97/Annabels_2_842f94c806_bfb48f2e97.svg</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Invitation only</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>Privileged access; Member experiences &amp; events; Community; Included member benefits</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>https://annabels.co.uk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Zero Bond</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Zero Bond</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Bond Hospitality</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcT1GOsXSa2VYZkjB_ezGUDz61tRPScQqS6q0nMx4RgKu4vfaCnbFDoh7hs&amp;s=10</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>Privileged access; Community; Member experiences &amp; events</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>https://zerobondny.com/apply-for-membership/</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>The Supper Club</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>The Supper Club (now Helm)</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>https://mma.prnewswire.com/media/2794987/supper_club_Logo.jpg?w=300</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Business Customers; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Subscription</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>Community; Member experiences &amp; events; Privileged access</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>https://www.helmclub.co/</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Wine Access Michelin Club</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Wine Access</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>https://d3h1lg3ksw6i6b.cloudfront.net/media/image/2022/02/03/8f721ef882bc48ad93a33c92171094fa_wine+access+vertical+logo+030222.png</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Enthusiasts / Hobbyists; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>North America; Global</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Subscription</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Open registration</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>Member pricing; Included member benefits; External partner network; Privileged access</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>https://www.wineaccess.com/subscriptions/</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Gourmet Escapes Privilege Club</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Gourmet Escapes</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>https://gourmet-escapes.com/wp-content/uploads/2017/09/logo.png</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; Enthusiasts / Hobbyists</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Subscription</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>Open registration</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>Member pricing; External partner network; Included member benefits; Privileged access</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>https://www.gourmet-escapes.com/privilege-club/</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Yellowstone Club</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Yellowstone Club</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>CrossHarbor Capital Partners</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>https://yellowstoneclub.com/logo-dark.svg</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Leisure &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>Invitation only</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>Privileged access; Community; Member experiences &amp; events; Included member benefits</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>https://yellowstoneclub.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Neera (Al Habtoor City, Dubai)</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Neera Private Members Club</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Al Habtoor Group</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>https://neeradubai.com/images/neera/peacock-feather.png</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Premium / Luxury Customers; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>Application required</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>Included member benefits; Member experiences &amp; events; Privileged access; Community</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>https://neeradubai.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Capital Club Dubai</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Capital Club Dubai</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>https://capitalclubdubai.com/wp-content/uploads/2021/04/cropped-Fatma-Al-Mahmoud-04.png</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Business Customers; High-Value Customers</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>Invitation only</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>Privileged access; External partner network; Community; Member experiences &amp; events</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>https://capitalclubdubai.com/membership/</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Rotana DISCOVERY</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Rotana Hotels &amp; Resorts</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>https://cdb.rotana.com/rcnimagelib/nx_logo_w_10.png</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Hotels &amp; Hospitality</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Business Customers; International Customers</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Middle East; Africa</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>Open registration</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>Spend-based earning; Earned status; External partner network; Privileged access</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>https://www.rotana.com/rotanadiscovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Zomato Gold</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Zomato</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Eternal Limited</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>https://b.zmtcdn.com/data/o2_assets/a8d9789aef91b9ffbca4f613010bb8d21714487350.png</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Mass Market; Frequent Customers</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Subscription</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>Open registration</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>Member pricing; Included member benefits; Privileged access</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>https://www.zomato.com/gold</t>
         </is>
       </c>
     </row>

</xml_diff>